<commit_message>
feat: progress per-type efficiency trend charts + UI polish + garmin token fix
- Add 4 full-width efficiency trend charts in Progress section (per training type), with year/month resolution toggle
- Polish pass: semantic h2 headings, table scope attrs, focus-visible states, reduced-motion support
- Fix garmin_sup_tracker.py token storage to use garminconnect 0.3+ format
- Add openpyxl to requirements.txt
</commit_message>
<xml_diff>
--- a/ניתוח_אימוני_SUP_v5.xlsx
+++ b/ניתוח_אימוני_SUP_v5.xlsx
@@ -1460,7 +1460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" style="41" min="1" max="1"/>
@@ -3987,6 +3987,370 @@
       <c r="L49" s="28" t="inlineStr">
         <is>
           <t>59:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>12.06.2026</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>אירובי</t>
+        </is>
+      </c>
+      <c r="C50" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="E50" s="28" t="inlineStr">
+        <is>
+          <t>55:29</t>
+        </is>
+      </c>
+      <c r="F50" s="28" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G50" s="28" t="n">
+        <v>133</v>
+      </c>
+      <c r="H50" s="28" t="n">
+        <v>36</v>
+      </c>
+      <c r="I50" s="28" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="J50" s="28" t="inlineStr">
+        <is>
+          <t>43:48</t>
+        </is>
+      </c>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>0:01</t>
+        </is>
+      </c>
+      <c r="L50" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>17.06.2026</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>אירובי</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="n">
+        <v>9.529999999999999</v>
+      </c>
+      <c r="E51" s="28" t="inlineStr">
+        <is>
+          <t>1:17:13</t>
+        </is>
+      </c>
+      <c r="F51" s="28" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G51" s="28" t="n">
+        <v>138</v>
+      </c>
+      <c r="H51" s="28" t="n">
+        <v>37</v>
+      </c>
+      <c r="I51" s="28" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J51" s="28" t="inlineStr">
+        <is>
+          <t>57:32</t>
+        </is>
+      </c>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="L51" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>19.06.2026</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>טמפו</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D52" s="28" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="E52" s="28" t="inlineStr">
+        <is>
+          <t>1:15:03</t>
+        </is>
+      </c>
+      <c r="F52" s="28" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G52" s="28" t="n">
+        <v>141</v>
+      </c>
+      <c r="H52" s="28" t="n">
+        <v>38</v>
+      </c>
+      <c r="I52" s="28" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="J52" s="28" t="inlineStr">
+        <is>
+          <t>36:22</t>
+        </is>
+      </c>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>28:59</t>
+        </is>
+      </c>
+      <c r="L52" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>20.06.2026</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>אירובי ארוך</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="E53" s="28" t="inlineStr">
+        <is>
+          <t>1:54:31</t>
+        </is>
+      </c>
+      <c r="F53" s="28" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G53" s="28" t="n">
+        <v>137</v>
+      </c>
+      <c r="H53" s="28" t="n">
+        <v>38</v>
+      </c>
+      <c r="I53" s="28" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J53" s="28" t="inlineStr">
+        <is>
+          <t>1:47:47</t>
+        </is>
+      </c>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>0:13</t>
+        </is>
+      </c>
+      <c r="L53" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>טמפו</t>
+        </is>
+      </c>
+      <c r="C54" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D54" s="28" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="E54" s="28" t="inlineStr">
+        <is>
+          <t>1:15:38</t>
+        </is>
+      </c>
+      <c r="F54" s="28" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G54" s="28" t="n">
+        <v>139</v>
+      </c>
+      <c r="H54" s="28" t="n">
+        <v>38</v>
+      </c>
+      <c r="I54" s="28" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="J54" s="28" t="inlineStr">
+        <is>
+          <t>41:25</t>
+        </is>
+      </c>
+      <c r="K54" s="28" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="L54" s="28" t="inlineStr">
+        <is>
+          <t>0:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="inlineStr">
+        <is>
+          <t>24.06.2026</t>
+        </is>
+      </c>
+      <c r="B55" s="28" t="inlineStr">
+        <is>
+          <t>טמפו</t>
+        </is>
+      </c>
+      <c r="C55" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="E55" s="28" t="inlineStr">
+        <is>
+          <t>1:15:22</t>
+        </is>
+      </c>
+      <c r="F55" s="28" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G55" s="28" t="n">
+        <v>144</v>
+      </c>
+      <c r="H55" s="28" t="n">
+        <v>38</v>
+      </c>
+      <c r="I55" s="28" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="J55" s="28" t="inlineStr">
+        <is>
+          <t>43:49</t>
+        </is>
+      </c>
+      <c r="K55" s="28" t="inlineStr">
+        <is>
+          <t>30:00</t>
+        </is>
+      </c>
+      <c r="L55" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="27" t="inlineStr">
+        <is>
+          <t>26.06.2026</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>אירובי</t>
+        </is>
+      </c>
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>ים</t>
+        </is>
+      </c>
+      <c r="D56" s="28" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="E56" s="28" t="inlineStr">
+        <is>
+          <t>1:12:20</t>
+        </is>
+      </c>
+      <c r="F56" s="28" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G56" s="28" t="n">
+        <v>135</v>
+      </c>
+      <c r="H56" s="28" t="n">
+        <v>37</v>
+      </c>
+      <c r="I56" s="28" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J56" s="28" t="inlineStr">
+        <is>
+          <t>1:02:40</t>
+        </is>
+      </c>
+      <c r="K56" s="28" t="inlineStr">
+        <is>
+          <t>0:13</t>
+        </is>
+      </c>
+      <c r="L56" s="28" t="inlineStr">
+        <is>
+          <t>0:00</t>
         </is>
       </c>
     </row>

</xml_diff>